<commit_message>
Tone down assignment answers to a plainer applicant voice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UWKenbiWBWMSaA2JAdanb6
</commit_message>
<xml_diff>
--- a/WEB広告_課題回答.xlsx
+++ b/WEB広告_課題回答.xlsx
@@ -6007,7 +6007,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>－－メール件名－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－</a:t>
+            <a:t>－－メール件名－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6021,7 +6021,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>【毎朝コンシーラーで隠しているシミ、ありませんか？】</a:t>
+            <a:t>そのシミ、もしかして美容液が届いていないだけかも？</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6035,21 +6035,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「塗っても変わらない」には、ちゃんと理由がありました</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－</a:t>
+            <a:t>－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6074,21 +6060,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>こんにちは。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>北の快適工房 スキンケア担当の高橋です。</a:t>
+            <a:t>こんにちは！</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6127,7 +6099,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>毎朝メイクをするとき、</a:t>
+            <a:t>毎朝メイクのときに</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6141,7 +6113,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「ここだけ、どうしても隠れない」</a:t>
+            <a:t>「このシミだけはどうしても隠れない…」</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6155,7 +6127,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>というシミはありませんか？</a:t>
+            <a:t>というシミ、ありませんか？</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6180,7 +6152,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>ファンデーションを塗っても</a:t>
+            <a:t>ファンデを塗っても透けて見えるから、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6194,7 +6166,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>うっすら透けて見える。</a:t>
+            <a:t>コンシーラーを重ねて、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6208,21 +6180,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>だからコンシーラーを重ねる。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>厚塗りになって、夕方にはヨレてまた目立つ…。</a:t>
+            <a:t>夕方にはヨレてまた目立ってくる。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6247,7 +6205,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>実は私も、左の頬にある</a:t>
+            <a:t>私もほっぺたのシミがずっと気になっていて、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6261,7 +6219,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>10円玉くらいのシミが長年の悩みでした。</a:t>
+            <a:t>美白美容液やクリームをいろいろ試しましたが、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>正直あまり変わった感じがしませんでした。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6286,35 +6258,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>美白美容液も、シミ用のクリームも、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>口コミで評判のものは一通り試しました。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>でも、なかなか変化を感じられない。</a:t>
+            <a:t>でも、それには理由があったんです。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6339,7 +6283,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「年齢的にもう仕方ないのかな」</a:t>
+            <a:t>肌にはもともと、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6353,7 +6297,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>そう諦めかけていたんです。</a:t>
+            <a:t>外から物が入らないようにする</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>バリア機能があります。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6378,7 +6336,35 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>■なぜ「塗る美白」では変わらないのか？</a:t>
+            <a:t>なので、どんなにいい美白成分でも、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>表面に塗るだけだと</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>なかなか奥まで届かないんです。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6403,7 +6389,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>理由は、とてもシンプルでした。</a:t>
+            <a:t>しかも美容液は顔全体に塗るので、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>気になるシミに届く量はほんの少しだけ。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6428,7 +6428,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>私たちの肌には、</a:t>
+            <a:t>「塗っても変わらない」のは、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6442,7 +6442,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>外からの異物が入り込まないように</a:t>
+            <a:t>ケアが足りないからではなく、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6456,7 +6456,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>“バリア機能”が備わっています。</a:t>
+            <a:t>成分が届いていなかったからかもしれません。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6481,7 +6481,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>そのため、どんなに良い美白成分でも</a:t>
+            <a:t>かといって皮膚科のレーザーは、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6495,7 +6495,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>肌の表面に塗るだけでは</a:t>
+            <a:t>お金もかかるし、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6509,7 +6509,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>なかなか奥まで届きにくいんです。</a:t>
+            <a:t>かさぶたやテープも気になるし、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>何より顔にレーザーはちょっと怖いですよね。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6534,7 +6548,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>しかも、美容液は顔全体に塗るもの。</a:t>
+            <a:t>そこでおすすめしたいのが</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6548,21 +6562,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>本当に気になる“あのシミ”に届く量は、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>実はほんのわずかしかありません。</a:t>
+            <a:t>「シミスポットパッチ」です！</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6587,7 +6587,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「塗っても変わらない」のは、</a:t>
+            <a:t>シミスポットパッチは、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6601,7 +6601,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>あなたのお手入れが足りないからではなく、</a:t>
+            <a:t>美白成分を細い“針”の形に固めた</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6615,7 +6615,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>そもそも成分が届いていなかったからかもしれないのです。</a:t>
+            <a:t>シミ専用のパッチです。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6640,7 +6640,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>とはいえ、皮膚科のレーザーは</a:t>
+            <a:t>使い方はとっても簡単で、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6654,35 +6654,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>費用もかかるし、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>かさぶたやテープで人目も気になる。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>何より「顔にレーザー」は少し怖いですよね。</a:t>
+            <a:t>夜、気になるシミの上に貼って寝るだけ。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6707,7 +6679,35 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>■そこで生まれたのが「シミスポットパッチ」です</a:t>
+            <a:t>貼ると細い針がシミの角質層まで刺さって、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>寝ている間に溶けて</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>美白成分を直接届けてくれます。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6732,7 +6732,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>シミスポットパッチは、</a:t>
+            <a:t>「塗る」のではなく「刺して届ける」から、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6746,35 +6746,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>美白有効成分とヒアルロン酸を</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>極細の“針”の形に固めた、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>“刺す”シミ集中ケアです。</a:t>
+            <a:t>今までの美白ケアとは全然ちがうんです。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6799,35 +6771,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>使い方は、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>夜のスキンケアの最後に</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>気になるシミの上に貼って寝るだけ。</a:t>
+            <a:t>しかも、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6852,7 +6796,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>貼ると、極細の針が</a:t>
+            <a:t>・気になるシミにだけピンポイントで貼れる</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6866,7 +6810,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>シミの角質層まで直接刺さり、</a:t>
+            <a:t>・朝ははがすだけなので毎日続けやすい</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6880,21 +6824,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>寝ている間にじわじわと溶けて</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>美白成分を届けます。</a:t>
+            <a:t>・家でできて、レーザーみたいなダウンタイムもない</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6919,35 +6849,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「塗る」のではなく「刺して届ける」。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>だから、今までの美白ケアとは</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>アプローチがまったく違うんです。</a:t>
+            <a:t>と、いいところばかり。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6972,7 +6874,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>■シミスポットパッチが選ばれる3つの理由</a:t>
+            <a:t>針と聞くと痛そうですが、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>貼るときにチクッとするくらいなので安心してください。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -6997,7 +6913,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>（1）成分が“届く”</a:t>
+            <a:t>シミのもとになるメラニンは、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7011,7 +6927,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>針そのものが美白成分でできているから、</a:t>
+            <a:t>紫外線を浴びるたびに毎日作られています。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7025,7 +6941,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>表面で流れ落ちることなく、</a:t>
+            <a:t>「そのうちやろう」と思っている間にも</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7039,7 +6955,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>角質層まで直接届けられます。</a:t>
+            <a:t>どんどんたまっていってしまいます。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7064,35 +6980,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>（2）気になるシミだけを“狙える”</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>シミに合わせた小さなパッチなので、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>「このシミ」にだけ成分を集中させられます。</a:t>
+            <a:t>だからこそ、気になった今がチャンスです！</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7117,7 +7005,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>（3）貼って寝るだけで“続けられる”</a:t>
+            <a:t>今なら初めての方限定で</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7131,7 +7019,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>朝ははがすだけ。</a:t>
+            <a:t>お得な特別価格で試せます。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7145,7 +7033,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>手間が増えないから、無理なく毎晩続けられます。</a:t>
+            <a:t>もし肌に合わなかったら全額返金保証もついているので、</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>試してみない手はないと思います！</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7170,7 +7072,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>「針」と聞くと痛そうに思うかもしれませんが、</a:t>
+            <a:t>毎朝コンシーラーを重ねる生活、</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7184,49 +7086,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>貼るときにチクッとする程度。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>北の快適工房の“刺す化粧品”は、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>シリーズ累計で数千万枚以上ご愛用いただいている</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>実績のある技術です。</a:t>
+            <a:t>今日で終わりにしませんか？</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7251,7 +7111,21 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>■シミは、待ってくれません</a:t>
+            <a:t>▼シミスポットパッチの詳細はこちら</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>https://（商品ページURL）</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -7276,417 +7150,7 @@
               <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>紫外線を浴びるたびに、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>メラニンは毎日つくられ続けています。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>「そのうち対策しよう」と</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>先延ばしにしている間にも、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>シミのもとは少しずつ積み重なっていきます。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>だからこそ、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>気になった“今日”が始めどきです。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>今なら、初めての方限定で</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>特別価格でお試しいただけます。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>さらに、万が一お肌に合わなかった場合は</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>全額返金保証つき。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>試すリスクはありません。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>毎朝、鏡の前でため息をつく日々を、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>今日で終わりにしませんか？</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>▼シミスポットパッチの詳細・特別価格はこちら</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>https://（商品ページURL）</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>※初回特別価格は数量限定のため、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>予定数に達し次第終了となります。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" altLang="ja-JP" sz="1050">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－－</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>追伸</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>コンシーラーを重ねなくてもいい朝は、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>想像以上に気持ちが軽くなります。</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>まずは一番気になる“あのシミ”から、</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="ja-JP" altLang="ja-JP" sz="1050">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:ea typeface="游ゴシック" panose="020B0400000000000000" pitchFamily="50" charset="-128"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>今夜はじめてみてください。</a:t>
+            <a:t>※特別価格は数に限りがあるので、なくなり次第終了です。</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -8071,73 +7535,70 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A38" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
 ▼平均より多くタップされた理由
-・《いいね！が止まらない》「SNSで火がついて大人気」「1500万枚が完売」という話題性・社会的証明のワードが並び、「今みんなが買っている物を自分だけ知らないのは損」という気持ちを刺激している。
-・文末が「〜化粧品とは？」と答えを伏せた問いかけになっており、商品名も用途も書かれていないため、「何だろう？」という純粋な好奇心でタップさせている。
-・画像がインスタグラムの投稿画面風で、企業の広告ではなく一般ユーザーの口コミ・流行のように見える。SmartNewsのニュース見出しの並びの中でも広告っぽさが薄く、記事感覚でタップされやすい。
-・「40代女性に大人気」と年齢を入れることで、40代のユーザーが「自分と同世代で流行っているもの」として目を止めやすい。
+「いいね！が止まらない」「1500万枚が完売」など、みんなが買っている感じの言葉が多くて、流行っているなら知っておきたいと思わせるからだと思います。
+また最後が「〜化粧品とは？」になっていて商品名が書いていないので、何の化粧品なのか気になってタップしてしまうと思います。
+画像もインスタの投稿みたいになっていて、広告っぽくなく普通の口コミに見えるのもタップされやすい理由だと思いました。
 ▼購入に至らなかった理由
-・タップの動機が「何が流行っているのか知りたい」という野次馬的な好奇心であり、「目元のシワ・乾燥をどうにかしたい」という悩み（＝購入動機）を広告の段階で一切想起させていない。そのため目元に悩みのない人や悩みの弱い人まで大量にタップし、遷移先で目元用パッチだと分かった瞬間に「自分には関係ない」と離脱している。
-・広告で期待させたもの（なぜSNSでバズったのか・どんな面白い商品なのか）と、遷移先ページの内容（目元のエイジングケア商品の説明）にズレがあり、クリック時の期待がページ内で回収されていない。
-・広告から「誰の・どんな悩みを・どう解決する商品か」が全く伝わらないため、ページを読み始めた時点で購入意欲がゼロからのスタートになる。
-・「40代女性に大人気」と書いているのに画像には若い女性が写っており、本来のターゲットである40代以上の女性が自分ごと化しにくい。
-・「マイクロニードル（針）」という商品特性についても、広告で事前に期待させていないため、ページで初めて知り「針を刺すのは怖い」という不安が先に立ちやすい。</t>
+タップした人の多くは「何が流行ってるんだろう？」という興味だけでタップしていて、目元のシワに悩んでいる人ばかりではなかったからだと思います。
+広告には何の悩みに使う商品か書いていないので、ページを開いて目元用のパッチだと分かった時点で「自分には関係ないな」と思って閉じてしまったのではないかと思います。
+あと「40代女性に大人気」と書いてあるのに画像は若い女性なので、40代の人が自分向けだと感じにくいのも原因だと思いました。</t>
         </is>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A39" s="50"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A40" s="50"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A41" s="50"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A42" s="50"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A43" s="50"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A44" s="50"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A45" s="50"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A46" s="50"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A47" s="50"/>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A48" s="50"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A49" s="50"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A50" s="50"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A51" s="50"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A52" s="50"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A53" s="50"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A54" s="50"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.5" ht="27.5" customHeight="1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A55" s="50"/>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.5">
@@ -8155,76 +7616,73 @@
         <v>76</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A59" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
 ▼変更後のテキストと画像のイメージをできるだけ具体的に記載してください
-【テキスト】（全角33文字）
+【テキスト】
 40代の目元の乾燥小ジワ問題。
 貼って寝る【刺すヒアルロン酸】が話題
 【画像】
-・インスタ投稿風のレイアウトと「いいね」の数は残し、写っている人物を40代の女性に変更。
-・パジャマ姿の40代女性が、目の下に半月型のパッチを貼って眠りにつく直前の写真をメインにする。
-・右下に丸い拡大窓を置き、パッチ表面の「ヒアルロン酸でできた極細の針」のイラストを表示し、「ヒアルロン酸を針状に固めた」と短い説明を入れる。
-・左上に「シリーズ累計1500万枚突破」のアイコンを小さく残す。
+インスタ投稿風のデザインといいねの数はそのまま残して、写っている人を40代くらいの女性に変えます。
+女性が目の下にパッチを貼って寝る前の写真にして、端に「累計1500万枚突破」と小さく入れます。
 ▼そのように変更する理由
-・元広告のタップ率の高さを生んでいる「SNSで話題」「1500万枚」「インスタ投稿風」といった話題性・社会的証明の要素は残し、タップ率は大きく落とさないようにする。
-・その上で「40代」「目元の乾燥小ジワ」と悩みを明示し、悩みを持つ見込み客だけがタップするよう絞り込む。冷やかしのタップを減らし、タップ後の購入率を上げる狙い。
-・「貼って寝るだけ」「刺すヒアルロン酸」で商品のカテゴリーと独自性（マイクロニードル）を事前に伝え、遷移先ページで「これのことか」と期待が回収される流れにする。針の存在を広告で前向きな新しさとして見せておくことで、ページで初めて知って不安になることも防ぐ。
-・人物を40代にすることで、ターゲットが「自分と同じ世代の人が使っている」と自分ごと化しやすくする。</t>
+今の広告はタップはされているので、「話題になっている感じ」やインスタ風の画像は残したほうがいいと思いました。
+その上で「40代の目元の乾燥小ジワ」と悩みをはっきり書くことで、本当に悩んでいる人がタップしてくれるようにしました。
+また「貼って寝る」「刺すヒアルロン酸」と何の商品かを少し見せておくことで、ページを開いたときに「思っていたのと違う」とならないようにしました。</t>
         </is>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A60" s="50"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A61" s="50"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A62" s="50"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A63" s="50"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A64" s="50"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A65" s="50"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A66" s="50"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A67" s="50"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A68" s="50"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A69" s="50"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A70" s="50"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A71" s="50"/>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A72" s="50"/>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A73" s="50"/>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A74" s="50"/>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A75" s="50"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.5" ht="25.39" customHeight="1">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A76" s="50"/>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.5">
@@ -8255,71 +7713,68 @@
         <v>78</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A107" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
 ▼ほぼタップされなかった理由
-・「ヒアロディープパッチ公式サイト」「北の快適工房がお届けする」と、商品名・企業名・公式サイトであることが前面に出ており、ひと目で「企業の宣伝」と分かる。ニュースを読みに来ているSmartNewsのユーザーにとっては、記事の中で浮いて読み飛ばされる。
-・商品を知らない人には「ヒアロディープパッチ」という名前が何の商品なのか分からず、誰の・どんな悩みを解決するのかが伝わらない（目元用であることすら分からない）。
-・「翌朝ルンルン気分に」は抽象的なイメージ表現で、具体的なベネフィットや意外性がなく、続きを知りたいという好奇心も生まれない。
-・画像も商品パッケージと「プレミアムナイトケアに」の文字が中心のイメージ広告的なもので、目を止める驚きや自分ごと化の要素がない。
+「公式サイト」「北の快適工房がお届けする」と書いてあって、ひと目で会社の宣伝だと分かってしまうからだと思います。ニュースを見ている途中だと、宣伝っぽいものは読み飛ばしてしまうと思います。
+また「ヒアロディープパッチ」という名前だけでは何の商品なのか分からず、「翌朝ルンルン気分に」もどう良いのかが伝わりにくいと思いました。
 ▼タップした人はほぼ全員が購入した理由
-・広告の情報量が商品説明に寄っているため、「ヒアルロン酸マイクロニードルのパッチ」と商品内容を理解した上で、なおかつ興味を持った人（もともと商品を知っている人・目元ケアの意識が高い人）だけがタップしている。つまり購入意欲の高い人だけが選別されている。
-・広告（公式サイト・商品名・パッケージ画像）と遷移先の公式ページの内容が完全に一致しており、期待とのギャップがない。
-・遷移先が公式の販売ページのため、商品説明から購入までの導線が短く、迷わず購入できる。</t>
+広告に商品名や商品の内容がそのまま書いてあるので、タップした人は最初からこの商品を知っていたり、目元ケアに興味がある人だけだったからだと思います。
+広告とページの内容も同じなので、イメージとのズレがなくそのまま購入したのだと思います。</t>
         </is>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A108" s="50"/>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A109" s="50"/>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A110" s="50"/>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A111" s="50"/>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A112" s="50"/>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A113" s="50"/>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A114" s="50"/>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A115" s="50"/>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A116" s="50"/>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A117" s="50"/>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A118" s="50"/>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A119" s="50"/>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A120" s="50"/>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A121" s="50"/>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A122" s="50"/>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A123" s="50"/>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.5" ht="21.17" customHeight="1">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A124" s="50"/>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.5">
@@ -8337,75 +7792,73 @@
         <v>76</v>
       </c>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A128" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
 ▼変更後のテキストと画像のイメージをできるだけ具体的に記載してください
-【テキスト】（全角32文字）
+【テキスト】
 目元の小ジワに「刺す」ケア？
 ヒアルロン酸の針が寝ている間に溶ける
 【画像】
-・目の下にパッチを貼って眠っている40〜50代女性の目元のアップ写真をメインにする。
-・その横に丸い拡大窓を置き、パッチの表面に並んだ極細の針（ヒアルロン酸でできた針）のイラストと、その針が肌の上で溶けていく様子を3コマで表示する。
-・パッケージ画像は右下に小さく残す程度にし、「公式サイト」「プレミアムナイトケア」の文字は外す。
+目の下にパッチを貼って寝ている女性の目元のアップにして、横にパッチの針の部分を拡大したイラストを入れます。
+商品のパッケージは右下に小さく入れるくらいにします。
 ▼そのように変更する理由
-・現在の広告は購入率が非常に高いので、「ヒアルロン酸のマイクロニードルを貼って寝る商品」という商品の中身はそのまま伝え、遷移先の公式ページとの一貫性を保つ（購入率を落とさない）。
-・その上で、タップ率が低い原因だった「企業の宣伝感」「誰の何の悩みか分からない」「好奇心が湧かない」を解消する。「目元の小ジワに」で悩みを明示して該当者の目を止め、「刺す」ケア？という意外性のある言葉と問いかけで「どういうこと？」という好奇心を生み、タップを促す。
-・「ヒアルロン酸の針が寝ている間に溶ける」で、針でも痛くなさそう・寝ている間に勝手にケアされるという具体的なベネフィットを伝え、興味をそのまま購入意欲につなげる。
-・画像も商品パッケージ中心から「使っているシーン＋仕組みの図解」に変え、ニュースの見出しの中でも目を引きつつ、ひと目で商品の新しさが分かるようにする。</t>
+今の広告は買う人の割合が高いので、ヒアルロン酸の針の商品だということは変えずに伝えるようにしました。
+ただそれだけだとタップされないので、「目元の小ジワに」と悩みを書いて、「刺す」ケア？と少し気になる言い方にしました。
+画像も商品パッケージだけより、使っているところが分かる方が目に止まりやすいと思いました。</t>
         </is>
       </c>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A129" s="50"/>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A130" s="50"/>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A131" s="50"/>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A132" s="50"/>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A133" s="50"/>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A134" s="50"/>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A135" s="50"/>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A136" s="50"/>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A137" s="50"/>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A138" s="50"/>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A139" s="50"/>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A140" s="50"/>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A141" s="50"/>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A142" s="50"/>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A143" s="50"/>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A144" s="50"/>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.5" ht="24.33" customHeight="1">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A145" s="50"/>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.5">
@@ -8770,83 +8223,69 @@
         <v>114</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A83" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
-【作成した広告】
-テキスト（全角32文字）：まぶたが重くて二重が消えた方へ／塗った瞬間ピンッ！まぶた専用ジェル
-画像（1200×628）：左に引き上がるまぶたのイラスト、右に「上まぶたの重さ・たるみ感に」「まぶた専用」「塗った瞬間キュッと引き締め美容ジェル」
-【ターゲット】
-40〜60代の女性で、年齢とともに上まぶたが重く下がってきて、二重の幅が狭くなった・二重が消えた、アイラインが引きにくい、目が小さく見える、と感じている人。SmartNewsの主要ユーザーである中高年層とも一致する。
-【テキストの意図】
-・SmartNewsのユーザーは広告を見に来ているのではなく、ニュースを流し読みしている。そのため1行目（15文字）だけで「自分のことだ」と気づかせる必要があると考え、「まぶたが重くて二重が消えた」という、ターゲットが日常的に鏡で感じている具体的な症状を冒頭に置いた。「たるみ」という抽象的な言葉よりも、本人が実感している現象を言い当てた方が自分ごと化しやすい。
-・「〜方へ」と呼びかけることで、該当する人に向けた記事であると思わせ、該当しない人のタップを減らして購入につながる人に絞り込む。
-・2行目では「塗った瞬間ピンッ！」と即効性の体感を擬音で伝えた。遷移先ページでは被膜によって塗ってすぐハリを感じられることが最大の特長として語られているため、広告で期待させた「すぐ変化を感じたい」という欲求がページで回収され、購入につながる。
-・「まぶた専用」は、アイクリームを目元全体に塗る程度しかしていない人にとって「まぶただけのケア用品があるのか」という意外性になり、同時に「専用だから効きそう」という期待を生む。
-【画像の意図】
-・ビフォーアフター写真やLPの画像は使えないため、イラストで「まぶたが上に引き上がる」矢印を見せ、テキストの「ピンッ！」と視覚的に連動させた。
-・右側に「まぶた専用」を最も大きく帯で配置し、小さな表示面でも商品の独自性がひと目で伝わるようにした。
-・「上まぶたの重さ・たるみ感に」で誰向けかを、「塗った瞬間キュッと引き締め」で何が起こるかを画像内でも補足し、テキストと画像のどちらを先に見ても内容が伝わるようにした。
-・ニュース記事の写真の中で浮きすぎないよう、肌なじみの良いピンクベージュ系の配色にして、エイジングケアの上品さと清潔感を出した。
-・使用感の表現には「※イメージです。使用感には個人差があります。」と注記を入れ、誇大な表現にならないよう配慮した。
-【遷移先ページとのつながり】
-広告で「まぶたの重さ・二重が消えた悩み」と「塗った瞬間の引き上げ感」に期待させ、記事風ページでまぶたが下がる原因と、まぶた専用・即効性の被膜という仕組みを読んで納得し、続けて使うことで本来のハリをケアできると知って公式ページで注文する、という流れを想定して作成した。</t>
+ターゲットは、年齢でまぶたが下がってきて「二重の幅がせまくなった」「目が小さくなった気がする」と感じている40〜60代の女性にしました。
+SmartNewsを見ている人はニュースを読みに来ているので、広告をじっくり見ないと思います。なので1行目で「まぶたが重くて二重が消えた」と、鏡を見て実際に感じていることをそのまま書いて、自分のことだと気づいてもらえるようにしました。「たるみ」よりも、二重が消えたと書いた方が分かりやすいと思いました。
+2行目の「塗った瞬間ピンッ！」は、ページの中で塗ってすぐハリを感じられることが一番の特長として書かれていたので、そこに期待してタップしてもらえるようにしました。「まぶた専用」は、まぶただけのケア商品はあまり聞かないので、気になってもらえると思って入れました。
+画像はビフォーアフターやLPの画像が使えないので、まぶたが上がる矢印のイラストにして、テキストの「ピンッ！」と合わせました。「まぶた専用」を一番大きく入れて、小さく表示されても何の商品か分かるようにしました。色はニュースの中で浮きすぎないように、肌に近いピンクベージュにしました。</t>
         </is>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A84" s="55"/>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A85" s="55"/>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A86" s="55"/>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A87" s="55"/>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A88" s="55"/>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A89" s="55"/>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A90" s="55"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A91" s="55"/>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A92" s="55"/>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A93" s="55"/>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A94" s="55"/>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A95" s="55"/>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A96" s="55"/>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A97" s="55"/>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A98" s="55"/>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A99" s="55"/>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A100" s="55"/>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.5" ht="39.05" customHeight="1">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A101" s="55"/>
     </row>
     <row r="102" spans="1:1" ht="16.5" x14ac:dyDescent="0.5">
@@ -11181,7 +10620,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.5" ht="107.0" customHeight="1">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.5" ht="90.5" customHeight="1">
       <c r="A32" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">【着眼元（仮）】
@@ -11194,15 +10633,15 @@
       <c r="B32" s="57"/>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">・「足の爪が白く濁る」という、自分の爪の見た目そのものを言い当てた症状の言葉にパッと目が止まって、（爪の色が気になっている人は、その言葉だけで自分の足の爪が頭に浮かぶ。）
-・かつ同時に、「NG習慣」という“自分もやっているかもしれない”と不安になる言葉にパッと目が止まって、</t>
+          <t xml:space="preserve">・「足の爪が白く濁る」という部分にパッと目が止まって、（自分の爪の色が気になっている人は、この言葉で自分の足の爪を思い出す。）
+・かつ「NG習慣」という言葉で、自分もやっているかもと思って目が止まって、</t>
         </is>
       </c>
       <c r="D32" s="57"/>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">・「足の爪が白く濁って分厚い」という症状の言葉でパッと目を止めさせて、（爪水虫という病名を知らない人・認めたくない人でも、症状を言い当てられれば自分の足の爪が頭に浮かび、目が止まる。）
-・かつ同時に、「〇〇問題。」というニュース見出しのようなフレーズで、広告ではなく記事として目を止めさせて、</t>
+          <t xml:space="preserve">・「足の爪が白く濁って分厚い」という症状の言葉でパッと目を止めさせて、（爪水虫と言われるとドキッとするけど、症状なら自分の爪を思い浮かべやすい。）
+・かつ「〜問題。」というニュースっぽい言い方で、広告っぽくなく目を止めさせて、</t>
         </is>
       </c>
       <c r="F32" s="57"/>
@@ -11226,13 +10665,13 @@
       <c r="B34" s="57"/>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">爪の濁りに心当たりがある人は、その原因が自分の普段の習慣にあると言われることで自分ごと化でき、かつ「3選」と答えがすぐに読めそうなことで、全文を読もうという気持ちになり、</t>
+          <t xml:space="preserve">自分の爪の濁りの原因が普段の習慣にあると言われて気になったのと、「3選」なのですぐ読めそうだと思ったので、全文読もうという気持ちになり、</t>
         </is>
       </c>
       <c r="D34" s="57"/>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">「白く濁る」だけでなく「分厚い」まで、爪水虫に悩む人が実際に感じている症状を具体的に言い当てることで、“まさに自分のことだ”と自分ごと化をより強めて、全文を読ませる気持ちにさせて、</t>
+          <t xml:space="preserve">「白く濁る」だけでなく「分厚い」まで書いて、まさに自分の爪のことだと思わせて、全文読ませる気持ちにさせて、</t>
         </is>
       </c>
       <c r="F34" s="57"/>
@@ -11251,18 +10690,18 @@
       <c r="F35" s="57"/>
       <c r="G35" s="60"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.5" ht="74.0" customHeight="1">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.5" ht="57.5" customHeight="1">
       <c r="A36" s="60"/>
       <c r="B36" s="57"/>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">普段何気なくしていることが爪の濁りの原因になっているかもしれないという驚きと、このまま放っておくとまずいのではという焦りの気持ちになって、</t>
+          <t xml:space="preserve">いつもしていることが原因かもしれないという驚きと、このままだとまずいかもという気持ちになって、</t>
         </is>
       </c>
       <c r="D36" s="57"/>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">「爪専用の薬用ジェル」というあまり聞かない言葉から、皮膚用の水虫薬では届きにくかった爪に専用で対処できそうという期待を感じさせつつ、「塗るだけで殺菌」から手軽に続けられそうという気持ちにさせて、</t>
+          <t xml:space="preserve">「爪専用の薬用ジェル」というあまり聞かない言葉から、爪に専用のものがあるんだという意外性と、塗るだけなら簡単に続けられそうという気持ちにさせて、</t>
         </is>
       </c>
       <c r="F36" s="57"/>
@@ -11286,13 +10725,13 @@
       <c r="B38" s="58"/>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">自分がNG習慣をしていないかの確認と、正しい対処法を求めてクリックした</t>
+          <t xml:space="preserve">自分がNG習慣をしていないかと、正しい対処法を知りたくてクリックした</t>
         </is>
       </c>
       <c r="D38" s="58"/>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">画像も相まって、爪専用の薬用ジェルの詳細（なぜ爪に使えるのか・どう使うのか）を求めてクリックさせる</t>
+          <t xml:space="preserve">画像も相まって、爪専用の薬用ジェルがどんな商品なのかを知りたくてクリックさせる</t>
         </is>
       </c>
       <c r="F38" s="58"/>
@@ -18260,64 +17699,60 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A13" s="110" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
-【ターゲット】
-40〜50代の女性で、頬やこめかみなどに濃く目立つシミが数個あり、毎朝コンシーラーで隠している人。美白美容液やシミ対策のクリームをいくつも試してきたが「塗っても変わらない」と感じており、皮膚科のレーザー治療も検討したことはあるものの、費用・かさぶたやテープなどのダウンタイム・痛みへの不安から踏み切れていない人。
-【設定理由】
-・顔全体のくすみではなく「ここにあるこのシミ」という一点の悩みを持つ人ほど、毎日鏡やメイクのたびに意識しており、悩みが深く、解決にお金を払う意欲が高い。
-・本商品は気になるシミにピンポイントで貼るパッチであり、顔全体に塗る美白美容液ではなく「特定のシミだけを集中ケアしたい」というニーズに最も合致する。
-・塗る美白ケアをすでに試して効果を実感できていない人には、「塗るのではなく、成分を固めた針で直接届ける」という本商品の仕組みが、これまでとの明確な違いとして響きやすい。
-・レーザーに踏み切れない層に対しては、「自宅で・貼って寝るだけ・ダウンタイムなし・手頃な価格」という代替手段として提案できる。
-・40〜50代はシミが濃く目立ち始める年代であり、スマートフォンでYahoo! JAPANのニュースを日常的に見ている層とも重なる。</t>
+40〜50代の女性で、頬などに目立つシミがあって毎朝コンシーラーで隠している人にしました。
+理由は、顔全体のくすみより「このシミが気になる」という人の方が、毎日鏡を見るたびに気になっていて、悩みが強いと思ったからです。
+また、美白美容液を使ってもあまり変わらなかった人や、皮膚科のレーザーは高いし怖くて行けない人にとって、貼って寝るだけのパッチはちょうどいいと思いました。
+シミに直接貼る商品なので、顔全体より「一か所のシミ」に悩んでいる人に合っていると思います。</t>
         </is>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A14" s="50"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A15" s="50"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A16" s="50"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A17" s="50"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A18" s="50"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A19" s="50"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A20" s="50"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A21" s="50"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A22" s="50"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A23" s="50"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A24" s="50"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A25" s="50"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A26" s="50"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A27" s="50"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.5" ht="21.44" customHeight="1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A28" s="50"/>
     </row>
     <row r="29" spans="1:1" s="19" customFormat="1" x14ac:dyDescent="0.5">
@@ -18335,65 +17770,62 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A32" s="111" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
-【強み①：美白有効成分を「針」にして、シミの角質層まで直接届ける】
-一般的な美白美容液やクリームは肌表面に塗るため、肌のバリア機能に阻まれて成分が届きにくく、洗顔やタオルで落ちてしまうものも多い。本商品は美白有効成分とヒアルロン酸を極細の針状に固めたマイクロニードルで、針が角質層に刺さってから溶け、成分を内側から直接届けられる。「塗っても変わらなかった」というターゲットの不満に対する明確な答えになる。
-【強み②：気になるシミ一点に、ピンポイントで集中ケアできる】
-顔全体に塗る美白ケアは、シミの部分に届く成分はごく一部。本商品はシミの大きさに合わせた小さなパッチを、気になるシミの上にだけ貼れるため、成分をそのシミに集中させられる。「このシミをどうにかしたい」というターゲットのニーズにそのまま応えられる。
-【強み③：貼って寝るだけ。自宅でできて、ダウンタイムもない】
-夜のスキンケアの最後に貼って寝て、朝はがすだけ。毎日の手間が増えず、寝ている間に針が溶けて浸透するので、ケアを「続けられる」。皮膚科のレーザーのような高額な費用、通院、かさぶた・テープ生活、痛みへの不安がなく、人に知られずに自宅でケアできる。
-【強み④：「刺す化粧品」としての実績と安心感】
-北の快適工房のマイクロニードル化粧品「ディープパッチシリーズ」は累計で数千万枚の販売実績があり、刺すといってもチクッとする程度で痛みはほとんどない。初めての「針」への不安を、実績で払拭できる。
-※広告表現に落とし込む際の軸は①（届く）と②（ピンポイント）とし、③④は不安解消・後押しの要素として使う想定です。</t>
+①美白成分を針にして、シミに直接届けられること
+美容液などは肌の表面に塗るだけなので成分が届きにくいですが、この商品は美白成分でできた細い針が刺さって中で溶けるので、塗るより届きやすいと思います。「塗っても変わらなかった」と思っている人に響くと思いました。
+②気になるシミだけにピンポイントで使えること
+顔全体に塗るものではなく、気になるシミの上にだけ貼れるので、そのシミを集中してケアできます。
+③貼って寝るだけで簡単なこと
+夜貼って朝はがすだけなので、面倒くさがりな人でも続けやすいです。レーザーと違って家でできて、かさぶたなどもないのも強みだと思います。</t>
         </is>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A33" s="50"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A34" s="50"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A35" s="50"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A36" s="50"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A37" s="50"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A38" s="50"/>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A39" s="50"/>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A40" s="50"/>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A41" s="50"/>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A42" s="50"/>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A43" s="50"/>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A44" s="50"/>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A45" s="50"/>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A46" s="50"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.5" ht="27.38" customHeight="1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A47" s="50"/>
     </row>
     <row r="48" spans="1:1" s="19" customFormat="1" x14ac:dyDescent="0.5">
@@ -18411,38 +17843,35 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A51" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">＜回答欄＞
 ①塗る美白で届かないシミに、“刺す”という選択。
 ②そのシミ、塗るより「刺して」届ける。
-③レーザーは怖い。でも、このシミは諦めたくない。貼って寝るだけのシミ集中ケア。
-④美白成分の“針”が、寝ている間にシミの角質層まで。
-⑤コンシーラーで隠す毎朝を、今日で終わりに。
-※「美白」は、メラニンの生成を抑え、シミ・そばかすを防ぐことを指します。</t>
+③レーザーは怖いけど、シミはあきらめたくない人へ。貼って寝るだけのシミケア。</t>
         </is>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A52" s="50"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A53" s="50"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A54" s="50"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A55" s="50"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A56" s="50"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A57" s="50"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.5" ht="19.12" customHeight="1">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.5" ht="24" customHeight="1">
       <c r="A58" s="50"/>
     </row>
     <row r="59" spans="1:1" s="19" customFormat="1" x14ac:dyDescent="0.5">

</xml_diff>